<commit_message>
Map Asana and Adaptive project states to the approved ServiceNow states
ServiceNow project states (implementation team): Open, Investigating,
Work in Progress, Closed Complete, Pending. Asana Not Started -> Pending,
Started/Scoping -> Investigating, In Progress/Delayed -> Work in Progress,
On Hold -> Pending, blank -> Pending; Completed/Cancelled stay out of the
in-flight load. Delayed and On Hold keep the source status as a
description line. Adaptive On Hold -> Pending for consistency.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/mapping/ServiceNow_SPM_Migration_Mapping.xlsx
+++ b/mapping/ServiceNow_SPM_Migration_Mapping.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Project Fields'!$A$1:$L$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Project Task Fields'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Value Maps'!$A$1:$E$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Value Maps'!$A$1:$E$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Unmapped Source Fields'!$A$1:$D$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Category'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sites'!$A$1:$A$26</definedName>
@@ -3391,7 +3391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>confirm</t>
         </is>
       </c>
     </row>
@@ -3473,12 +3473,12 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Investigating</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>confirm</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>confirm</t>
         </is>
       </c>
     </row>
@@ -3527,12 +3527,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Work in Progress</t>
+          <t>Work in Progress (+ description line 'Asana status: Delayed')</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>confirm</t>
         </is>
       </c>
     </row>
@@ -3554,12 +3554,12 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>On Hold</t>
+          <t>Pending (+ description line 'Asana status: On Hold')</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>confirm</t>
         </is>
       </c>
     </row>
@@ -3581,10 +3581,14 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>(not migrated - in-flight scope)</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
+          <t>Closed Complete (only if completed projects are migrated; in-flight scope skips them)</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -3604,7 +3608,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>(not migrated)</t>
+          <t>(not migrated - no cancelled/closed-incomplete state)</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
@@ -3612,56 +3616,52 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>State (Adaptive)</t>
+          <t>State (Asana)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>(blank)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Work in Progress</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>confirm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>State (Adaptive)</t>
+          <t>State (Asana)</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>(ServiceNow)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>On Hold</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>On Hold</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>-3</t>
-        </is>
-      </c>
+          <t>Open - not used by Asana</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -3676,15 +3676,19 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Requested</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>(loads as Demand)</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr"/>
+          <t>Work in Progress</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -3699,15 +3703,19 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>On Hold</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>(loads as Demand)</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr"/>
+          <t>Pending (+ description line 'Adaptive state: On Hold')</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -3722,12 +3730,12 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Requested</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>(not migrated - in-flight scope)</t>
+          <t>(loads as Demand)</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
@@ -3745,12 +3753,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Cancelled</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>(not migrated)</t>
+          <t>(loads as Demand)</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
@@ -3758,56 +3766,48 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Task State</t>
+          <t>State (Adaptive)</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Asana (task)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>-5</t>
-        </is>
-      </c>
+          <t>(not migrated - in-flight scope)</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Task State</t>
+          <t>State (Adaptive)</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Asana (task)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Cancelled</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Work in Progress</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>(not migrated)</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -3822,108 +3822,120 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Closed Complete</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>confirm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Funding</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Asana / Adaptive</t>
+          <t>Asana (task)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>OpEx / Opex</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Funding Type: Opex required | Expense type: Opex</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr"/>
+          <t>Work in Progress</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Funding</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Asana / Adaptive</t>
+          <t>Asana (task)</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>CapEx / Capex</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Funding Type: Capex required | Expense type: Capex</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr"/>
+          <t>Closed Complete</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Investment Class</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Asana (task)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>(blank)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Change</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr"/>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Investment Class</t>
+          <t>Funding</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Asana / Adaptive</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Annual Program</t>
+          <t>OpEx / Opex</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Funding Type: Opex required | Expense type: Opex</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr"/>
@@ -3931,22 +3943,22 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Investment Class</t>
+          <t>Funding</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Asana / Adaptive</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Project/Annual Program</t>
+          <t>CapEx / Capex</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Change</t>
+          <t>Funding Type: Capex required | Expense type: Capex</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr"/>
@@ -3954,22 +3966,22 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Investment Class</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>On Target / On Plan</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Change</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr"/>
@@ -3977,22 +3989,22 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Investment Class</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Needs Attention</t>
+          <t>Annual Program</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Run</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr"/>
@@ -4000,22 +4012,22 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Investment Class</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>In Trouble</t>
+          <t>Project/Annual Program</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Change</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr"/>
@@ -4023,7 +4035,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -4033,12 +4045,12 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Initiation</t>
+          <t>On Target / On Plan</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>(ServiceNow phase value - not in data model file)</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr"/>
@@ -4046,7 +4058,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -4056,12 +4068,12 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Discovery &amp; Design</t>
+          <t>Needs Attention</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>(ServiceNow phase value - not in data model file)</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr"/>
@@ -4069,7 +4081,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -4079,12 +4091,12 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Execution</t>
+          <t>In Trouble</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>(ServiceNow phase value - not in data model file)</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr"/>
@@ -4102,7 +4114,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Close Out</t>
+          <t>Initiation</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -4115,7 +4127,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -4125,24 +4137,20 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Construction/Relocation</t>
+          <t>Discovery &amp; Design</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Construction/relocation</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>construction_relocation</t>
-        </is>
-      </c>
+          <t>(ServiceNow phase value - not in data model file)</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -4152,24 +4160,20 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Onboarding (new Provider group - no construction)</t>
+          <t>Execution</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Onboarding (new Provider group - no construction)</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>onboarding</t>
-        </is>
-      </c>
+          <t>(ServiceNow phase value - not in data model file)</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -4179,19 +4183,15 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Close Out</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Application</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>application</t>
-        </is>
-      </c>
+          <t>(ServiceNow phase value - not in data model file)</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -4206,17 +4206,17 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Construction/Relocation</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Construction/relocation</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>epic</t>
+          <t>construction_relocation</t>
         </is>
       </c>
     </row>
@@ -4233,17 +4233,17 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>GHC - all non RSFH work</t>
+          <t>Onboarding (new Provider group - no construction)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>GHC - all not FSFH work</t>
+          <t>Onboarding (new Provider group - no construction)</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>ghc</t>
+          <t>onboarding</t>
         </is>
       </c>
     </row>
@@ -4260,17 +4260,17 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>application</t>
         </is>
       </c>
     </row>
@@ -4287,17 +4287,17 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Medical Group</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Medical Group</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>medical_group</t>
+          <t>epic</t>
         </is>
       </c>
     </row>
@@ -4314,17 +4314,17 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Revenue Cycle (includes Ensemble requests</t>
+          <t>GHC - all non RSFH work</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Revenue Cycle (includes Ensemble requests)</t>
+          <t>GHC - all not FSFH work</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>revenue_cycle</t>
+          <t>ghc</t>
         </is>
       </c>
     </row>
@@ -4341,17 +4341,17 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>RSFH</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>RSFH</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>rsfh</t>
+          <t>infrastructure</t>
         </is>
       </c>
     </row>
@@ -4368,17 +4368,17 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Medical Group</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Medical Group</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>security</t>
+          <t>medical_group</t>
         </is>
       </c>
     </row>
@@ -4395,29 +4395,29 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>Revenue Cycle (includes Ensemble requests</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>Revenue Cycle (includes Ensemble requests)</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>urgent care</t>
+          <t>revenue_cycle</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Asana)</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -4439,48 +4439,56 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Asana)</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>BSMH</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>(no matching choice in the data model)</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr"/>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Asana)</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>GBS</t>
+          <t>Urgent Care</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>(no matching choice in the data model)</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr"/>
+          <t>Urgent Care</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>urgent care</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -4495,35 +4503,39 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>External Partners</t>
+          <t>RSFH</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>(no matching choice in the data model)</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr"/>
+          <t>RSFH</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>rsfh</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Asana)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Advantus Health Partners</t>
+          <t>BSMH</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Advantus Health Partners</t>
+          <t>(no matching choice in the data model)</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr"/>
@@ -4531,22 +4543,22 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Asana)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Affiliate</t>
+          <t>GBS</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Affiliate</t>
+          <t>(no matching choice in the data model)</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr"/>
@@ -4554,22 +4566,22 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Asana)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Chesapeake (GHC)</t>
+          <t>External Partners</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Chesapeake (GHC)</t>
+          <t>(no matching choice in the data model)</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr"/>
@@ -4587,12 +4599,12 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Cincinnati</t>
+          <t>Advantus Health Partners</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Cincinnati</t>
+          <t>Advantus Health Partners</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr"/>
@@ -4610,12 +4622,12 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Conduit Health</t>
+          <t>Affiliate</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Conduit Health</t>
+          <t>Affiliate</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr"/>
@@ -4633,12 +4645,12 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Covenant (GHC)</t>
+          <t>Chesapeake (GHC)</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Covenant (GHC)</t>
+          <t>Chesapeake (GHC)</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr"/>
@@ -4656,12 +4668,12 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Ensemble</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Ensemble</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr"/>
@@ -4679,12 +4691,12 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Conduit Health</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Conduit Health</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr"/>
@@ -4702,12 +4714,12 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Global Business Services (GBS)</t>
+          <t>Covenant (GHC)</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Global Business Services (GBS)</t>
+          <t>Covenant (GHC)</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr"/>
@@ -4725,12 +4737,12 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Greenville</t>
+          <t>Ensemble</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Greenville</t>
+          <t>Ensemble</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr"/>
@@ -4748,12 +4760,12 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Hampton Roads</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Hampton Roads</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr"/>
@@ -4771,12 +4783,12 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Harness Health Partners</t>
+          <t>Global Business Services (GBS)</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Harness Health Partners</t>
+          <t>Global Business Services (GBS)</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr"/>
@@ -4794,12 +4806,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Home Office</t>
+          <t>Greenville</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Home Office</t>
+          <t>Greenville</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr"/>
@@ -4817,12 +4829,12 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Hampton Roads</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Hampton Roads</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr"/>
@@ -4840,12 +4852,12 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Harness Health Partners</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Harness Health Partners</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr"/>
@@ -4863,12 +4875,12 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Home Office</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Home Office</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr"/>
@@ -4886,12 +4898,12 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Lorain</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Lorain</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr"/>
@@ -4909,12 +4921,12 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Nationwide (GHC)</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Nationwide (GHC)</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr"/>
@@ -4932,12 +4944,12 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr"/>
@@ -4955,12 +4967,12 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Roper St. Francis Healthcare</t>
+          <t>Lorain</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Roper St. Francis Healthcare</t>
+          <t>Lorain</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr"/>
@@ -4978,12 +4990,12 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Shelter Arms (GHC)</t>
+          <t>Nationwide (GHC)</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Shelter Arms (GHC)</t>
+          <t>Nationwide (GHC)</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr"/>
@@ -5001,12 +5013,12 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr"/>
@@ -5024,12 +5036,12 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Roper St. Francis Healthcare</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Roper St. Francis Healthcare</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr"/>
@@ -5047,12 +5059,12 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Wyandot (GHC)</t>
+          <t>Shelter Arms (GHC)</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>Wyandot (GHC)</t>
+          <t>Shelter Arms (GHC)</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr"/>
@@ -5070,18 +5082,87 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
+          <t>Springfield</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>Springfield</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Wyandot (GHC)</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>Wyandot (GHC)</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
           <t>Youngstown</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D72" s="6" t="inlineStr">
         <is>
           <t>Youngstown</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr"/>
+      <c r="E72" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E69"/>
+  <autoFilter ref="A1:E72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Map Asana and Adaptive task states to the six approved project task states
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/mapping/ServiceNow_SPM_Migration_Mapping.xlsx
+++ b/mapping/ServiceNow_SPM_Migration_Mapping.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Project Fields'!$A$1:$L$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Project Task Fields'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Value Maps'!$A$1:$E$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Value Maps'!$A$1:$E$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Unmapped Source Fields'!$A$1:$D$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Category'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sites'!$A$1:$A$26</definedName>
@@ -3391,7 +3391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3849,12 +3849,12 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Started/Scoping</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Work in Progress</t>
+          <t>Investigating</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -3876,12 +3876,12 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Closed Complete</t>
+          <t>Work in Progress</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -3903,12 +3903,12 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>(blank)</t>
+          <t>Delayed</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Work in Progress (+ description line 'Asana status: Delayed')</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -3920,229 +3920,265 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Funding</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Asana / Adaptive</t>
+          <t>Asana (task)</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>OpEx / Opex</t>
+          <t>On Hold</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Funding Type: Opex required | Expense type: Opex</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr"/>
+          <t>Pending (+ description line 'Asana status: On Hold')</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Funding</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Asana / Adaptive</t>
+          <t>Asana (task)</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>CapEx / Capex</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Funding Type: Capex required | Expense type: Capex</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr"/>
+          <t>Closed Complete</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Investment Class</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Asana (task)</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Cancelled</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Change</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr"/>
+          <t>Closed Incomplete</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Investment Class</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Asana (task)</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Annual Program</t>
+          <t>(blank)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr"/>
+          <t>Pending; Closed Complete if the task has a Completed At date</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Investment Class</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive (task)</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Project/Annual Program</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Change</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr"/>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Adaptive (task)</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>On Target / On Plan</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Green</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr"/>
+          <t>Work in Progress</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Adaptive (task)</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Needs Attention</t>
+          <t>On Hold</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr"/>
+          <t>Pending (+ description line 'Adaptive state: On Hold')</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Adaptive (task)</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>In Trouble</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr"/>
+          <t>Closed Complete</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Adaptive (task)</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Initiation</t>
+          <t>Cancelled</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>(ServiceNow phase value - not in data model file)</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr"/>
+          <t>Closed Incomplete</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Task State</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>(ServiceNow)</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Discovery &amp; Design</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>(ServiceNow phase value - not in data model file)</t>
+          <t>Open - not used by either source</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr"/>
@@ -4150,22 +4186,22 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Funding</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana / Adaptive</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Execution</t>
+          <t>OpEx / Opex</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>(ServiceNow phase value - not in data model file)</t>
+          <t>Funding Type: Opex required | Expense type: Opex</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr"/>
@@ -4173,22 +4209,22 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Funding</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana / Adaptive</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Close Out</t>
+          <t>CapEx / Capex</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>(ServiceNow phase value - not in data model file)</t>
+          <t>Funding Type: Capex required | Expense type: Capex</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr"/>
@@ -4196,88 +4232,76 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Investment Class</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Construction/Relocation</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Construction/relocation</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>construction_relocation</t>
-        </is>
-      </c>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Investment Class</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Onboarding (new Provider group - no construction)</t>
+          <t>Annual Program</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Onboarding (new Provider group - no construction)</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>onboarding</t>
-        </is>
-      </c>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Investment Class</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Adaptive</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Project/Annual Program</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Application</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>application</t>
-        </is>
-      </c>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -4287,24 +4311,20 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>On Target / On Plan</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>epic</t>
-        </is>
-      </c>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -4314,24 +4334,20 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>GHC - all non RSFH work</t>
+          <t>Needs Attention</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>GHC - all not FSFH work</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>ghc</t>
-        </is>
-      </c>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -4341,24 +4357,20 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>In Trouble</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr">
-        <is>
-          <t>infrastructure</t>
-        </is>
-      </c>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -4368,24 +4380,20 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Medical Group</t>
+          <t>Initiation</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Medical Group</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>medical_group</t>
-        </is>
-      </c>
+          <t>(ServiceNow phase value - not in data model file)</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -4395,24 +4403,20 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Revenue Cycle (includes Ensemble requests</t>
+          <t>Discovery &amp; Design</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Revenue Cycle (includes Ensemble requests)</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>revenue_cycle</t>
-        </is>
-      </c>
+          <t>(ServiceNow phase value - not in data model file)</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -4422,24 +4426,20 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>RSFH</t>
+          <t>Execution</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>RSFH</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>rsfh</t>
-        </is>
-      </c>
+          <t>(ServiceNow phase value - not in data model file)</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Adaptive)</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
@@ -4449,19 +4449,15 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Close Out</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>security</t>
-        </is>
-      </c>
+          <t>(ServiceNow phase value - not in data model file)</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -4476,296 +4472,336 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>Construction/Relocation</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>Construction/relocation</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>urgent care</t>
+          <t>construction_relocation</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Asana)</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>RSFH</t>
+          <t>Onboarding (new Provider group - no construction)</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>RSFH</t>
+          <t>Onboarding (new Provider group - no construction)</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>rsfh</t>
+          <t>onboarding</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Asana)</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>BSMH</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>(no matching choice in the data model)</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr"/>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>application</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Asana)</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>GBS</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>(no matching choice in the data model)</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr"/>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Business Category (Asana)</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>External Partners</t>
+          <t>GHC - all non RSFH work</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>(no matching choice in the data model)</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr"/>
+          <t>GHC - all not FSFH work</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>ghc</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Advantus Health Partners</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Advantus Health Partners</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr"/>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Affiliate</t>
+          <t>Medical Group</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Affiliate</t>
-        </is>
-      </c>
-      <c r="E49" s="6" t="inlineStr"/>
+          <t>Medical Group</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>medical_group</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Chesapeake (GHC)</t>
+          <t>Revenue Cycle (includes Ensemble requests</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Chesapeake (GHC)</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr"/>
+          <t>Revenue Cycle (includes Ensemble requests)</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>revenue_cycle</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Cincinnati</t>
+          <t>RSFH</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Cincinnati</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr"/>
+          <t>RSFH</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>rsfh</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Conduit Health</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Conduit Health</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr"/>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Adaptive)</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Covenant (GHC)</t>
+          <t>Urgent Care</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Covenant (GHC)</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr"/>
+          <t>Urgent Care</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>urgent care</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Asana)</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Ensemble</t>
+          <t>RSFH</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Ensemble</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr"/>
+          <t>RSFH</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>rsfh</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Asana)</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>BSMH</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>(no matching choice in the data model)</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr"/>
@@ -4773,22 +4809,22 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Asana)</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Global Business Services (GBS)</t>
+          <t>GBS</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Global Business Services (GBS)</t>
+          <t>(no matching choice in the data model)</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr"/>
@@ -4796,22 +4832,22 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>Sites</t>
+          <t>Business Category (Asana)</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Adaptive (Region)</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Greenville</t>
+          <t>External Partners</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Greenville</t>
+          <t>(no matching choice in the data model)</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr"/>
@@ -4829,12 +4865,12 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Hampton Roads</t>
+          <t>Advantus Health Partners</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Hampton Roads</t>
+          <t>Advantus Health Partners</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr"/>
@@ -4852,12 +4888,12 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Harness Health Partners</t>
+          <t>Affiliate</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Harness Health Partners</t>
+          <t>Affiliate</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr"/>
@@ -4875,12 +4911,12 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Home Office</t>
+          <t>Chesapeake (GHC)</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Home Office</t>
+          <t>Chesapeake (GHC)</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr"/>
@@ -4898,12 +4934,12 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr"/>
@@ -4921,12 +4957,12 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Conduit Health</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Conduit Health</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr"/>
@@ -4944,12 +4980,12 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Covenant (GHC)</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Covenant (GHC)</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr"/>
@@ -4967,12 +5003,12 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Lorain</t>
+          <t>Ensemble</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Lorain</t>
+          <t>Ensemble</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr"/>
@@ -4990,12 +5026,12 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Nationwide (GHC)</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Nationwide (GHC)</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr"/>
@@ -5013,12 +5049,12 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Global Business Services (GBS)</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Global Business Services (GBS)</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr"/>
@@ -5036,12 +5072,12 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Roper St. Francis Healthcare</t>
+          <t>Greenville</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Roper St. Francis Healthcare</t>
+          <t>Greenville</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr"/>
@@ -5059,12 +5095,12 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Shelter Arms (GHC)</t>
+          <t>Hampton Roads</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>Shelter Arms (GHC)</t>
+          <t>Hampton Roads</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr"/>
@@ -5082,12 +5118,12 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Harness Health Partners</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Harness Health Partners</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr"/>
@@ -5105,12 +5141,12 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Home Office</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Home Office</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr"/>
@@ -5128,12 +5164,12 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Wyandot (GHC)</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Wyandot (GHC)</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr"/>
@@ -5151,18 +5187,248 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
+          <t>Kentucky</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>Kentucky</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Lima</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>Lima</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Lorain</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>Lorain</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Nationwide (GHC)</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>Nationwide (GHC)</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Roper St. Francis Healthcare</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Roper St. Francis Healthcare</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Shelter Arms (GHC)</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>Shelter Arms (GHC)</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Springfield</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>Springfield</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Wyandot (GHC)</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Wyandot (GHC)</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive (Region)</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
           <t>Youngstown</t>
         </is>
       </c>
-      <c r="D72" s="6" t="inlineStr">
+      <c r="D82" s="6" t="inlineStr">
         <is>
           <t>Youngstown</t>
         </is>
       </c>
-      <c r="E72" s="6" t="inlineStr"/>
+      <c r="E82" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E72"/>
+  <autoFilter ref="A1:E82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>